<commit_message>
Update pricing and billing usage model
</commit_message>
<xml_diff>
--- a/strategy/pricing/pricing-model-codex-20260619/Arcova_Pricing_Model.xlsx
+++ b/strategy/pricing/pricing-model-codex-20260619/Arcova_Pricing_Model.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R32ea503df0124282"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Credits" sheetId="2" r:id="R61ad59bf225d4c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Model" sheetId="3" r:id="Rbfdee94a505a4325"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Entitlements" sheetId="4" r:id="Rfd2c1f6dd86f469b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Model" sheetId="5" r:id="R2c26613306d34de3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Touchpoints" sheetId="6" r:id="R97608b63250a4bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R5dfd608df9c749e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Rules" sheetId="8" r:id="R5a38adb4156a4d88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R0d91c441181148bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" r:id="R8b3b5e0d80e1497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="11" r:id="Rc788480fbc124cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R9e5321fbc2b340f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Credits" sheetId="2" r:id="R7052761d594e4a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Model" sheetId="3" r:id="R65ec501a6cec4ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Entitlements" sheetId="4" r:id="R3115d88fc7274b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Model" sheetId="5" r:id="R9120ff0a162c49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Touchpoints" sheetId="6" r:id="R64c9756975694639"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R1752e155a4ae45e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Rules" sheetId="8" r:id="R81dc423578404739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R32a64cebe1ab4a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" r:id="R19cfa8579af44570"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="11" r:id="Rfd55368581ce4985"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1323,7 +1323,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08e643e1c6794a9d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7c7cf72f8c054205"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -7564,14 +7564,14 @@
       </x:c>
       <x:c r="B5" s="197" t="n">
         <x:f>'Tier Model'!N6</x:f>
-        <x:v>0.6003355704697987</x:v>
+        <x:v>0.5998322147651006</x:v>
       </x:c>
       <x:c r="C5" s="151" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="151" t="n">
         <x:f>B5-C5</x:f>
-        <x:v>0.6003355704697987</x:v>
+        <x:v>0.5998322147651006</x:v>
       </x:c>
       <x:c r="E5" s="151" t="n">
         <x:v>0</x:v>
@@ -7609,14 +7609,14 @@
       </x:c>
       <x:c r="B6" s="199" t="n">
         <x:f>'Tier Model'!N7</x:f>
-        <x:v>0.627909887359199</x:v>
+        <x:v>0.6277221526908635</x:v>
       </x:c>
       <x:c r="C6" s="154" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="154" t="n">
         <x:f>B6-C6</x:f>
-        <x:v>0.627909887359199</x:v>
+        <x:v>0.6277221526908635</x:v>
       </x:c>
       <x:c r="E6" s="154" t="n">
         <x:v>0</x:v>
@@ -13416,11 +13416,11 @@
       </x:c>
       <x:c r="J6" s="216" t="n">
         <x:f>'Tier Model'!M6</x:f>
-        <x:v>59.55</x:v>
+        <x:v>59.625</x:v>
       </x:c>
       <x:c r="K6" s="197" t="n">
         <x:f>'Tier Model'!N6</x:f>
-        <x:v>0.6003355704697987</x:v>
+        <x:v>0.5998322147651006</x:v>
       </x:c>
       <x:c r="L6" s="217" t="n">
         <x:f>'Tier Model'!D6</x:f>
@@ -13446,7 +13446,7 @@
         <x:v>Starter</x:v>
       </x:c>
       <x:c r="B7" s="154" t="str">
-        <x:v>$149 / workspace / month · 2,000 credits · 5,000 active leads monitored monthly</x:v>
+        <x:v>$149 / workspace / month · 2,000 credits · 3 active ICPs · 5,000 active leads monitored monthly</x:v>
       </x:c>
       <x:c r="C7" s="154"/>
       <x:c r="D7" s="154"/>
@@ -13462,11 +13462,11 @@
       </x:c>
       <x:c r="J7" s="218" t="n">
         <x:f>'Tier Model'!M7</x:f>
-        <x:v>297.3</x:v>
+        <x:v>297.45000000000005</x:v>
       </x:c>
       <x:c r="K7" s="209" t="n">
         <x:f>'Tier Model'!N7</x:f>
-        <x:v>0.627909887359199</x:v>
+        <x:v>0.6277221526908635</x:v>
       </x:c>
       <x:c r="L7" s="219" t="n">
         <x:f>'Tier Model'!D7</x:f>
@@ -13492,7 +13492,7 @@
         <x:v>Growth</x:v>
       </x:c>
       <x:c r="B8" s="154" t="str">
-        <x:v>$799 / workspace / month · 8,000 credits · 10,000 active leads monitored weekly</x:v>
+        <x:v>$799 / workspace / month · 8,000 credits · 10 active ICPs · 10,000 active leads monitored weekly</x:v>
       </x:c>
       <x:c r="C8" s="154"/>
       <x:c r="D8" s="154"/>
@@ -13735,7 +13735,7 @@
       </x:c>
       <x:c r="C15" s="198" t="n">
         <x:f>'Action Credits'!D8</x:f>
-        <x:v>0.031000000000000003</x:v>
+        <x:v>0.0325</x:v>
       </x:c>
       <x:c r="D15" s="198" t="n">
         <x:f>B15/1000*100</x:f>
@@ -14182,7 +14182,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B27" s="154" t="str">
-        <x:v>A new ICP triggers free re-triage of non-enriched records and a free cached rescore of enriched records—not blanket provider enrichment.</x:v>
+        <x:v>Active ICPs are capped by plan: 1 on Free, 3 on Starter, 10 on Growth. Editing an existing ICP is free; adding another active ICP requires an available slot or upgrade.</x:v>
       </x:c>
       <x:c r="C27" s="154"/>
       <x:c r="D27" s="154"/>
@@ -19082,7 +19082,7 @@
     <x:mergeCell ref="B29:L29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1d7eae63724507"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45138e76feb4f64"/>
 </x:worksheet>
 </file>
 
@@ -19392,21 +19392,21 @@
         <x:v>User selects ranked lead / bulk queue</x:v>
       </x:c>
       <x:c r="C8" s="154" t="str">
-        <x:v>1.3 Apollo + Apify</x:v>
+        <x:v>1.3 Apollo + Apify + 30% ZB validation</x:v>
       </x:c>
       <x:c r="D8" s="166" t="n">
-        <x:f>Assumptions!C12*Assumptions!C11+Assumptions!C15</x:f>
-        <x:v>0.031000000000000003</x:v>
+        <x:f>'Assumptions'!C12*'Assumptions'!C11+'Assumptions'!C15+'Assumptions'!B29*'Assumptions'!C17</x:f>
+        <x:v>0.0325</x:v>
       </x:c>
       <x:c r="E8" s="167" t="n">
         <x:f>D8/Assumptions!B6</x:f>
-        <x:v>3.1</x:v>
+        <x:v>3.25</x:v>
       </x:c>
       <x:c r="F8" s="168" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="154" t="str">
-        <x:v>4 credits / contact+company lead</x:v>
+        <x:v>4 credits / contact+company lead; validation included when email returned</x:v>
       </x:c>
       <x:c r="H8" s="154" t="str">
         <x:v>No</x:v>
@@ -19415,7 +19415,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="J8" s="155" t="str">
-        <x:v>Use canonical company/person cache before provider call.</x:v>
+        <x:v>Includes ZeroBounce validation when an email is returned. Validation COGS is modeled as validation share x ZB unit cost.</x:v>
       </x:c>
       <x:c r="K8" s="138"/>
       <x:c r="L8" s="138"/>
@@ -19696,11 +19696,11 @@
       </x:c>
       <x:c r="D14" s="166" t="n">
         <x:f>D8</x:f>
-        <x:v>0.031000000000000003</x:v>
+        <x:v>0.0325</x:v>
       </x:c>
       <x:c r="E14" s="167" t="n">
         <x:f>D14/Assumptions!B6</x:f>
-        <x:v>3.1</x:v>
+        <x:v>3.25</x:v>
       </x:c>
       <x:c r="F14" s="168" t="n">
         <x:v>4</x:v>
@@ -19846,11 +19846,11 @@
       </x:c>
       <x:c r="D17" s="166" t="n">
         <x:f>D8</x:f>
-        <x:v>0.031000000000000003</x:v>
+        <x:v>0.0325</x:v>
       </x:c>
       <x:c r="E17" s="167" t="n">
         <x:f>D17/Assumptions!B6</x:f>
-        <x:v>3.1</x:v>
+        <x:v>3.25</x:v>
       </x:c>
       <x:c r="F17" s="168" t="n">
         <x:v>0</x:v>
@@ -25238,11 +25238,11 @@
       </x:c>
       <x:c r="L5" s="177" t="n">
         <x:f>D5*F5*Assumptions!C16+(D5*Assumptions!B27*'Action Credits'!D17)+Assumptions!B38</x:f>
-        <x:v>1.431</x:v>
+        <x:v>1.4325</x:v>
       </x:c>
       <x:c r="M5" s="177" t="n">
         <x:f>K5+L5</x:f>
-        <x:v>2.431</x:v>
+        <x:v>2.4325</x:v>
       </x:c>
       <x:c r="N5" s="178" t="str">
         <x:f>""</x:f>
@@ -25297,15 +25297,15 @@
       </x:c>
       <x:c r="L6" s="182" t="n">
         <x:f>D6*F6*Assumptions!C16+(D6*Assumptions!B27*'Action Credits'!D17)+Assumptions!B39</x:f>
-        <x:v>39.55</x:v>
+        <x:v>39.625</x:v>
       </x:c>
       <x:c r="M6" s="182" t="n">
         <x:f>K6+L6</x:f>
-        <x:v>59.55</x:v>
+        <x:v>59.625</x:v>
       </x:c>
       <x:c r="N6" s="183" t="n">
         <x:f>(B6-M6)/B6</x:f>
-        <x:v>0.6003355704697987</x:v>
+        <x:v>0.5998322147651006</x:v>
       </x:c>
       <x:c r="O6" s="138"/>
       <x:c r="P6" s="138"/>
@@ -25357,15 +25357,15 @@
       </x:c>
       <x:c r="L7" s="187" t="n">
         <x:f>D7*F7*Assumptions!C16+(D7*Assumptions!B27*'Action Credits'!D17)+Assumptions!B40</x:f>
-        <x:v>217.3</x:v>
+        <x:v>217.45000000000002</x:v>
       </x:c>
       <x:c r="M7" s="187" t="n">
         <x:f>K7+L7</x:f>
-        <x:v>297.3</x:v>
+        <x:v>297.45000000000005</x:v>
       </x:c>
       <x:c r="N7" s="188" t="n">
         <x:f>(B7-M7)/B7</x:f>
-        <x:v>0.627909887359199</x:v>
+        <x:v>0.6277221526908635</x:v>
       </x:c>
       <x:c r="O7" s="138"/>
       <x:c r="P7" s="138"/>
@@ -25843,8 +25843,12 @@
       <x:c r="Z21" s="138"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="138"/>
-      <x:c r="B22" s="138"/>
+      <x:c r="A22" s="138" t="str">
+        <x:v>Active ICPs</x:v>
+      </x:c>
+      <x:c r="B22" s="138" t="str">
+        <x:v>Free includes 1 active ICP; Starter includes 3; Growth includes 10. Purchased credits do not increase ICP capacity; editing an existing ICP does not consume another slot.</x:v>
+      </x:c>
       <x:c r="C22" s="138"/>
       <x:c r="D22" s="138"/>
       <x:c r="E22" s="138"/>
@@ -32103,12 +32107,24 @@
       <x:c r="Z31" s="138"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="138"/>
-      <x:c r="B32" s="138"/>
-      <x:c r="C32" s="138"/>
-      <x:c r="D32" s="138"/>
-      <x:c r="E32" s="138"/>
-      <x:c r="F32" s="138"/>
+      <x:c r="A32" s="138" t="str">
+        <x:v>Active ICP cap</x:v>
+      </x:c>
+      <x:c r="B32" s="138" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C32" s="138" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D32" s="138" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E32" s="138" t="str">
+        <x:v>saved active ICPs</x:v>
+      </x:c>
+      <x:c r="F32" s="138" t="str">
+        <x:v>Editing an existing ICP is free; creating another active ICP requires an available slot or a higher plan.</x:v>
+      </x:c>
       <x:c r="G32" s="138"/>
       <x:c r="H32" s="138"/>
       <x:c r="I32" s="138"/>
@@ -37583,7 +37599,7 @@
       </x:c>
       <x:c r="E22" s="198" t="n">
         <x:f>B22*'Action Credits'!D8</x:f>
-        <x:v>1.2400000000000002</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="F22" s="199" t="n">
         <x:f>IF($D$28=0,0,D22/$D$28)</x:f>
@@ -37857,7 +37873,7 @@
       </x:c>
       <x:c r="E28" s="202" t="n">
         <x:f>SUM(E21:E27)</x:f>
-        <x:v>11.450000000000001</x:v>
+        <x:v>11.51</x:v>
       </x:c>
       <x:c r="F28" s="201"/>
       <x:c r="G28" s="203"/>
@@ -49005,23 +49021,23 @@
       </x:c>
       <x:c r="B6" s="197" t="n">
         <x:f>(149-(2000*$A6*Assumptions!B6+B$5*Assumptions!C16+B$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.8167114093959731</x:v>
+        <x:v>0.8166107382550335</x:v>
       </x:c>
       <x:c r="C6" s="197" t="n">
         <x:f>(149-(2000*$A6*Assumptions!B6+C$5*Assumptions!C16+C$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7733221476510067</x:v>
+        <x:v>0.7730704697986577</x:v>
       </x:c>
       <x:c r="D6" s="197" t="n">
         <x:f>(149-(2000*$A6*Assumptions!B6+D$5*Assumptions!C16+D$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.701006711409396</x:v>
+        <x:v>0.700503355704698</x:v>
       </x:c>
       <x:c r="E6" s="197" t="n">
         <x:f>(149-(2000*$A6*Assumptions!B6+E$5*Assumptions!C16+E$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6286912751677852</x:v>
+        <x:v>0.6279362416107382</x:v>
       </x:c>
       <x:c r="F6" s="178" t="n">
         <x:f>(149-(2000*$A6*Assumptions!B6+F$5*Assumptions!C16+F$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5563758389261745</x:v>
+        <x:v>0.5553691275167785</x:v>
       </x:c>
       <x:c r="G6" s="138"/>
       <x:c r="H6" s="138"/>
@@ -49050,23 +49066,23 @@
       </x:c>
       <x:c r="B7" s="199" t="n">
         <x:f>(149-(2000*$A7*Assumptions!B6+B$5*Assumptions!C16+B$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7831543624161074</x:v>
+        <x:v>0.7830536912751678</x:v>
       </x:c>
       <x:c r="C7" s="199" t="n">
         <x:f>(149-(2000*$A7*Assumptions!B6+C$5*Assumptions!C16+C$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7397651006711409</x:v>
+        <x:v>0.739513422818792</x:v>
       </x:c>
       <x:c r="D7" s="199" t="n">
         <x:f>(149-(2000*$A7*Assumptions!B6+D$5*Assumptions!C16+D$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6674496644295302</x:v>
+        <x:v>0.6669463087248322</x:v>
       </x:c>
       <x:c r="E7" s="199" t="n">
         <x:f>(149-(2000*$A7*Assumptions!B6+E$5*Assumptions!C16+E$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5951342281879194</x:v>
+        <x:v>0.5943791946308725</x:v>
       </x:c>
       <x:c r="F7" s="183" t="n">
         <x:f>(149-(2000*$A7*Assumptions!B6+F$5*Assumptions!C16+F$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5228187919463088</x:v>
+        <x:v>0.5218120805369127</x:v>
       </x:c>
       <x:c r="G7" s="138"/>
       <x:c r="H7" s="138"/>
@@ -49095,23 +49111,23 @@
       </x:c>
       <x:c r="B8" s="199" t="n">
         <x:f>(149-(2000*$A8*Assumptions!B6+B$5*Assumptions!C16+B$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7495973154362416</x:v>
+        <x:v>0.7494966442953019</x:v>
       </x:c>
       <x:c r="C8" s="199" t="n">
         <x:f>(149-(2000*$A8*Assumptions!B6+C$5*Assumptions!C16+C$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7062080536912752</x:v>
+        <x:v>0.7059563758389261</x:v>
       </x:c>
       <x:c r="D8" s="199" t="n">
         <x:f>(149-(2000*$A8*Assumptions!B6+D$5*Assumptions!C16+D$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6338926174496644</x:v>
+        <x:v>0.6333892617449665</x:v>
       </x:c>
       <x:c r="E8" s="199" t="n">
         <x:f>(149-(2000*$A8*Assumptions!B6+E$5*Assumptions!C16+E$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5615771812080537</x:v>
+        <x:v>0.5608221476510067</x:v>
       </x:c>
       <x:c r="F8" s="183" t="n">
         <x:f>(149-(2000*$A8*Assumptions!B6+F$5*Assumptions!C16+F$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.489261744966443</x:v>
+        <x:v>0.48825503355704697</x:v>
       </x:c>
       <x:c r="G8" s="138"/>
       <x:c r="H8" s="138"/>
@@ -49140,23 +49156,23 @@
       </x:c>
       <x:c r="B9" s="199" t="n">
         <x:f>(149-(2000*$A9*Assumptions!B6+B$5*Assumptions!C16+B$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.7160402684563758</x:v>
+        <x:v>0.7159395973154362</x:v>
       </x:c>
       <x:c r="C9" s="199" t="n">
         <x:f>(149-(2000*$A9*Assumptions!B6+C$5*Assumptions!C16+C$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6726510067114093</x:v>
+        <x:v>0.6723993288590604</x:v>
       </x:c>
       <x:c r="D9" s="199" t="n">
         <x:f>(149-(2000*$A9*Assumptions!B6+D$5*Assumptions!C16+D$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6003355704697987</x:v>
+        <x:v>0.5998322147651006</x:v>
       </x:c>
       <x:c r="E9" s="199" t="n">
         <x:f>(149-(2000*$A9*Assumptions!B6+E$5*Assumptions!C16+E$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5280201342281879</x:v>
+        <x:v>0.527265100671141</x:v>
       </x:c>
       <x:c r="F9" s="183" t="n">
         <x:f>(149-(2000*$A9*Assumptions!B6+F$5*Assumptions!C16+F$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.4557046979865772</x:v>
+        <x:v>0.4546979865771812</x:v>
       </x:c>
       <x:c r="G9" s="138"/>
       <x:c r="H9" s="138"/>
@@ -49185,23 +49201,23 @@
       </x:c>
       <x:c r="B10" s="209" t="n">
         <x:f>(149-(2000*$A10*Assumptions!B6+B$5*Assumptions!C16+B$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6824832214765101</x:v>
+        <x:v>0.6823825503355705</x:v>
       </x:c>
       <x:c r="C10" s="209" t="n">
         <x:f>(149-(2000*$A10*Assumptions!B6+C$5*Assumptions!C16+C$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.6390939597315436</x:v>
+        <x:v>0.6388422818791947</x:v>
       </x:c>
       <x:c r="D10" s="209" t="n">
         <x:f>(149-(2000*$A10*Assumptions!B6+D$5*Assumptions!C16+D$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.5667785234899329</x:v>
+        <x:v>0.5662751677852349</x:v>
       </x:c>
       <x:c r="E10" s="209" t="n">
         <x:f>(149-(2000*$A10*Assumptions!B6+E$5*Assumptions!C16+E$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.4944630872483221</x:v>
+        <x:v>0.4937080536912752</x:v>
       </x:c>
       <x:c r="F10" s="188" t="n">
         <x:f>(149-(2000*$A10*Assumptions!B6+F$5*Assumptions!C16+F$5*Assumptions!B27*'Action Credits'!D17+Assumptions!B39))/149</x:f>
-        <x:v>0.4221476510067114</x:v>
+        <x:v>0.4211409395973154</x:v>
       </x:c>
       <x:c r="G10" s="138"/>
       <x:c r="H10" s="138"/>
@@ -49356,23 +49372,23 @@
       </x:c>
       <x:c r="B15" s="197" t="n">
         <x:f>(499-(8000*$A15*Assumptions!B6+B$14*Assumptions!B28*Assumptions!C16+B$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.7894288577154309</x:v>
+        <x:v>0.7893537074148297</x:v>
       </x:c>
       <x:c r="C15" s="197" t="n">
         <x:f>(499-(8000*$A15*Assumptions!B6+C$14*Assumptions!B28*Assumptions!C16+C$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.7011022044088177</x:v>
+        <x:v>0.7009519038076152</x:v>
       </x:c>
       <x:c r="D15" s="197" t="n">
         <x:f>(499-(8000*$A15*Assumptions!B6+D$14*Assumptions!B28*Assumptions!C16+D$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.6127755511022044</x:v>
+        <x:v>0.6125501002004008</x:v>
       </x:c>
       <x:c r="E15" s="197" t="n">
         <x:f>(499-(8000*$A15*Assumptions!B6+E$14*Assumptions!B28*Assumptions!C16+E$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.5244488977955911</x:v>
+        <x:v>0.5241482965931863</x:v>
       </x:c>
       <x:c r="F15" s="178" t="n">
         <x:f>(499-(8000*$A15*Assumptions!B6+F$14*Assumptions!B28*Assumptions!C16+F$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.34779559118236475</x:v>
+        <x:v>0.3473446893787575</x:v>
       </x:c>
       <x:c r="G15" s="138"/>
       <x:c r="H15" s="138"/>
@@ -49401,23 +49417,23 @@
       </x:c>
       <x:c r="B16" s="199" t="n">
         <x:f>(499-(8000*$A16*Assumptions!B6+B$14*Assumptions!B28*Assumptions!C16+B$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.7493486973947895</x:v>
+        <x:v>0.7492735470941884</x:v>
       </x:c>
       <x:c r="C16" s="199" t="n">
         <x:f>(499-(8000*$A16*Assumptions!B6+C$14*Assumptions!B28*Assumptions!C16+C$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.6610220440881764</x:v>
+        <x:v>0.6608717434869739</x:v>
       </x:c>
       <x:c r="D16" s="199" t="n">
         <x:f>(499-(8000*$A16*Assumptions!B6+D$14*Assumptions!B28*Assumptions!C16+D$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.5726953907815631</x:v>
+        <x:v>0.5724699398797596</x:v>
       </x:c>
       <x:c r="E16" s="199" t="n">
         <x:f>(499-(8000*$A16*Assumptions!B6+E$14*Assumptions!B28*Assumptions!C16+E$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.48436873747494985</x:v>
+        <x:v>0.484068136272545</x:v>
       </x:c>
       <x:c r="F16" s="183" t="n">
         <x:f>(499-(8000*$A16*Assumptions!B6+F$14*Assumptions!B28*Assumptions!C16+F$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.3077154308617235</x:v>
+        <x:v>0.3072645290581162</x:v>
       </x:c>
       <x:c r="G16" s="138"/>
       <x:c r="H16" s="138"/>
@@ -49446,23 +49462,23 @@
       </x:c>
       <x:c r="B17" s="199" t="n">
         <x:f>(499-(8000*$A17*Assumptions!B6+B$14*Assumptions!B28*Assumptions!C16+B$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.7092685370741482</x:v>
+        <x:v>0.709193386773547</x:v>
       </x:c>
       <x:c r="C17" s="199" t="n">
         <x:f>(499-(8000*$A17*Assumptions!B6+C$14*Assumptions!B28*Assumptions!C16+C$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.620941883767535</x:v>
+        <x:v>0.6207915831663327</x:v>
       </x:c>
       <x:c r="D17" s="199" t="n">
         <x:f>(499-(8000*$A17*Assumptions!B6+D$14*Assumptions!B28*Assumptions!C16+D$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.5326152304609219</x:v>
+        <x:v>0.5323897795591183</x:v>
       </x:c>
       <x:c r="E17" s="199" t="n">
         <x:f>(499-(8000*$A17*Assumptions!B6+E$14*Assumptions!B28*Assumptions!C16+E$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.4442885771543086</x:v>
+        <x:v>0.4439879759519037</x:v>
       </x:c>
       <x:c r="F17" s="183" t="n">
         <x:f>(499-(8000*$A17*Assumptions!B6+F$14*Assumptions!B28*Assumptions!C16+F$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.26763527054108216</x:v>
+        <x:v>0.2671843687374749</x:v>
       </x:c>
       <x:c r="G17" s="138"/>
       <x:c r="H17" s="138"/>
@@ -49491,23 +49507,23 @@
       </x:c>
       <x:c r="B18" s="199" t="n">
         <x:f>(499-(8000*$A18*Assumptions!B6+B$14*Assumptions!B28*Assumptions!C16+B$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.669188376753507</x:v>
+        <x:v>0.6691132264529058</x:v>
       </x:c>
       <x:c r="C18" s="199" t="n">
         <x:f>(499-(8000*$A18*Assumptions!B6+C$14*Assumptions!B28*Assumptions!C16+C$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.5808617234468937</x:v>
+        <x:v>0.5807114228456913</x:v>
       </x:c>
       <x:c r="D18" s="199" t="n">
         <x:f>(499-(8000*$A18*Assumptions!B6+D$14*Assumptions!B28*Assumptions!C16+D$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.4925350701402806</x:v>
+        <x:v>0.49230961923847694</x:v>
       </x:c>
       <x:c r="E18" s="199" t="n">
         <x:f>(499-(8000*$A18*Assumptions!B6+E$14*Assumptions!B28*Assumptions!C16+E$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.4042084168336673</x:v>
+        <x:v>0.40390781563126243</x:v>
       </x:c>
       <x:c r="F18" s="183" t="n">
         <x:f>(499-(8000*$A18*Assumptions!B6+F$14*Assumptions!B28*Assumptions!C16+F$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.2275551102204409</x:v>
+        <x:v>0.22710420841683365</x:v>
       </x:c>
       <x:c r="G18" s="138"/>
       <x:c r="H18" s="138"/>
@@ -49536,23 +49552,23 @@
       </x:c>
       <x:c r="B19" s="209" t="n">
         <x:f>(499-(8000*$A19*Assumptions!B6+B$14*Assumptions!B28*Assumptions!C16+B$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.6291082164328656</x:v>
+        <x:v>0.6290330661322645</x:v>
       </x:c>
       <x:c r="C19" s="209" t="n">
         <x:f>(499-(8000*$A19*Assumptions!B6+C$14*Assumptions!B28*Assumptions!C16+C$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.5407815631262525</x:v>
+        <x:v>0.54063126252505</x:v>
       </x:c>
       <x:c r="D19" s="209" t="n">
         <x:f>(499-(8000*$A19*Assumptions!B6+D$14*Assumptions!B28*Assumptions!C16+D$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.4524549098196392</x:v>
+        <x:v>0.4522294589178357</x:v>
       </x:c>
       <x:c r="E19" s="209" t="n">
         <x:f>(499-(8000*$A19*Assumptions!B6+E$14*Assumptions!B28*Assumptions!C16+E$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.36412825651302594</x:v>
+        <x:v>0.36382765531062117</x:v>
       </x:c>
       <x:c r="F19" s="188" t="n">
         <x:f>(499-(8000*$A19*Assumptions!B6+F$14*Assumptions!B28*Assumptions!C16+F$14*Assumptions!B27*'Action Credits'!D17+Assumptions!B40))/499</x:f>
-        <x:v>0.18747494989979963</x:v>
+        <x:v>0.18702404809619236</x:v>
       </x:c>
       <x:c r="G19" s="138"/>
       <x:c r="H19" s="138"/>
@@ -55299,12 +55315,24 @@
       <x:c r="Z16" s="138"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="138"/>
-      <x:c r="B17" s="138"/>
-      <x:c r="C17" s="138"/>
-      <x:c r="D17" s="138"/>
-      <x:c r="E17" s="138"/>
-      <x:c r="F17" s="138"/>
+      <x:c r="A17" s="138" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="B17" s="138" t="str">
+        <x:v>Active ICP capacity</x:v>
+      </x:c>
+      <x:c r="C17" s="138" t="str">
+        <x:v>Create ICP</x:v>
+      </x:c>
+      <x:c r="D17" s="138" t="str">
+        <x:v>No credits; workspace cap check</x:v>
+      </x:c>
+      <x:c r="E17" s="138" t="str">
+        <x:v>Free 1, Starter 3, Growth 10; edit/delete to manage slots</x:v>
+      </x:c>
+      <x:c r="F17" s="138" t="str">
+        <x:v>Server-side cap enforced; DB-level race guard not added</x:v>
+      </x:c>
       <x:c r="G17" s="138"/>
       <x:c r="H17" s="138"/>
       <x:c r="I17" s="138"/>

</xml_diff>